<commit_message>
Actualizacion automatica 2026-09-18 17:11 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2331" uniqueCount="614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2317" uniqueCount="614">
   <si>
     <t>Tablero Servicios y mantención</t>
   </si>
@@ -11636,7 +11636,7 @@
       </c>
       <c r="C176" s="6"/>
       <c r="D176" s="5">
-        <v>46277.13662217592</v>
+        <v>46245.57038168982</v>
       </c>
       <c r="E176" s="6" t="s">
         <v>562</v>
@@ -11676,9 +11676,7 @@
         <v>563</v>
       </c>
       <c r="R176" s="6"/>
-      <c r="S176" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S176" s="6"/>
       <c r="T176" s="6"/>
       <c r="U176" s="6"/>
     </row>
@@ -11691,7 +11689,7 @@
       </c>
       <c r="C177" s="11"/>
       <c r="D177" s="10">
-        <v>46277.13662469907</v>
+        <v>46245.57032159722</v>
       </c>
       <c r="E177" s="11" t="s">
         <v>565</v>
@@ -11731,9 +11729,7 @@
         <v>566</v>
       </c>
       <c r="R177" s="11"/>
-      <c r="S177" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S177" s="11"/>
       <c r="T177" s="11"/>
       <c r="U177" s="11"/>
     </row>
@@ -11746,7 +11742,7 @@
       </c>
       <c r="C178" s="6"/>
       <c r="D178" s="5">
-        <v>46277.13662829861</v>
+        <v>46245.570321747684</v>
       </c>
       <c r="E178" s="6" t="s">
         <v>565</v>
@@ -11786,9 +11782,7 @@
         <v>568</v>
       </c>
       <c r="R178" s="6"/>
-      <c r="S178" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S178" s="6"/>
       <c r="T178" s="6"/>
       <c r="U178" s="6"/>
     </row>
@@ -11801,7 +11795,7 @@
       </c>
       <c r="C179" s="11"/>
       <c r="D179" s="10">
-        <v>46277.13662234954</v>
+        <v>46245.57032184028</v>
       </c>
       <c r="E179" s="11" t="s">
         <v>565</v>
@@ -11841,9 +11835,7 @@
         <v>570</v>
       </c>
       <c r="R179" s="11"/>
-      <c r="S179" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S179" s="11"/>
       <c r="T179" s="11"/>
       <c r="U179" s="11"/>
     </row>
@@ -11856,7 +11848,7 @@
       </c>
       <c r="C180" s="6"/>
       <c r="D180" s="5">
-        <v>46277.136622129634</v>
+        <v>46245.57032194444</v>
       </c>
       <c r="E180" s="6" t="s">
         <v>572</v>
@@ -11896,9 +11888,7 @@
         <v>573</v>
       </c>
       <c r="R180" s="6"/>
-      <c r="S180" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S180" s="6"/>
       <c r="T180" s="6"/>
       <c r="U180" s="6"/>
     </row>
@@ -11911,7 +11901,7 @@
       </c>
       <c r="C181" s="11"/>
       <c r="D181" s="10">
-        <v>46277.136622453705</v>
+        <v>46245.570322025465</v>
       </c>
       <c r="E181" s="11" t="s">
         <v>572</v>
@@ -11951,9 +11941,7 @@
         <v>575</v>
       </c>
       <c r="R181" s="11"/>
-      <c r="S181" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S181" s="11"/>
       <c r="T181" s="11"/>
       <c r="U181" s="11"/>
     </row>
@@ -11966,7 +11954,7 @@
       </c>
       <c r="C182" s="6"/>
       <c r="D182" s="5">
-        <v>46277.136627604166</v>
+        <v>46245.57032210648</v>
       </c>
       <c r="E182" s="6" t="s">
         <v>572</v>
@@ -12006,9 +11994,7 @@
         <v>577</v>
       </c>
       <c r="R182" s="6"/>
-      <c r="S182" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S182" s="6"/>
       <c r="T182" s="6"/>
       <c r="U182" s="6"/>
     </row>
@@ -12021,7 +12007,7 @@
       </c>
       <c r="C183" s="11"/>
       <c r="D183" s="10">
-        <v>46277.13662239583</v>
+        <v>46245.5703221875</v>
       </c>
       <c r="E183" s="11" t="s">
         <v>572</v>
@@ -12061,9 +12047,7 @@
         <v>579</v>
       </c>
       <c r="R183" s="11"/>
-      <c r="S183" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S183" s="11"/>
       <c r="T183" s="11"/>
       <c r="U183" s="11"/>
     </row>
@@ -12076,7 +12060,7 @@
       </c>
       <c r="C184" s="6"/>
       <c r="D184" s="5">
-        <v>46277.1366231713</v>
+        <v>46245.57032229166</v>
       </c>
       <c r="E184" s="6" t="s">
         <v>572</v>
@@ -12116,9 +12100,7 @@
         <v>581</v>
       </c>
       <c r="R184" s="6"/>
-      <c r="S184" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S184" s="6"/>
       <c r="T184" s="6"/>
       <c r="U184" s="6"/>
     </row>
@@ -12131,7 +12113,7 @@
       </c>
       <c r="C185" s="11"/>
       <c r="D185" s="10">
-        <v>46277.1366240625</v>
+        <v>46245.57032237269</v>
       </c>
       <c r="E185" s="11" t="s">
         <v>572</v>
@@ -12171,9 +12153,7 @@
         <v>583</v>
       </c>
       <c r="R185" s="11"/>
-      <c r="S185" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S185" s="11"/>
       <c r="T185" s="11"/>
       <c r="U185" s="11"/>
     </row>
@@ -12186,7 +12166,7 @@
       </c>
       <c r="C186" s="6"/>
       <c r="D186" s="5">
-        <v>46277.136627604166</v>
+        <v>46245.57032246528</v>
       </c>
       <c r="E186" s="6" t="s">
         <v>572</v>
@@ -12226,9 +12206,7 @@
         <v>585</v>
       </c>
       <c r="R186" s="6"/>
-      <c r="S186" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S186" s="6"/>
       <c r="T186" s="6"/>
       <c r="U186" s="6"/>
     </row>
@@ -12241,7 +12219,7 @@
       </c>
       <c r="C187" s="11"/>
       <c r="D187" s="10">
-        <v>46277.136622164355</v>
+        <v>46245.570322534724</v>
       </c>
       <c r="E187" s="11" t="s">
         <v>572</v>
@@ -12281,9 +12259,7 @@
         <v>587</v>
       </c>
       <c r="R187" s="11"/>
-      <c r="S187" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S187" s="11"/>
       <c r="T187" s="11"/>
       <c r="U187" s="11"/>
     </row>
@@ -12296,7 +12272,7 @@
       </c>
       <c r="C188" s="6"/>
       <c r="D188" s="5">
-        <v>46277.136624861116</v>
+        <v>46245.57032261574</v>
       </c>
       <c r="E188" s="6" t="s">
         <v>572</v>
@@ -12336,9 +12312,7 @@
         <v>589</v>
       </c>
       <c r="R188" s="6"/>
-      <c r="S188" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S188" s="6"/>
       <c r="T188" s="6"/>
       <c r="U188" s="6"/>
     </row>
@@ -12351,7 +12325,7 @@
       </c>
       <c r="C189" s="11"/>
       <c r="D189" s="10">
-        <v>46277.13662228009</v>
+        <v>46245.57032271991</v>
       </c>
       <c r="E189" s="11" t="s">
         <v>572</v>
@@ -12391,9 +12365,7 @@
         <v>591</v>
       </c>
       <c r="R189" s="11"/>
-      <c r="S189" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S189" s="11"/>
       <c r="T189" s="11"/>
       <c r="U189" s="11"/>
     </row>

</xml_diff>